<commit_message>
Execute visual ChromeDriver session for 300 web test cases and export 5-sheet report
</commit_message>
<xml_diff>
--- a/selenium_test_suite/TestReports/PetOrb_Selenium_Test_Report.xlsx
+++ b/selenium_test_suite/TestReports/PetOrb_Selenium_Test_Report.xlsx
@@ -961,7 +961,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>4.72 s</t>
+          <t>4.71 s</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:58:15</t>
+          <t>2026-07-29 03:01:57</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -1522,7 +1522,7 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -1802,7 +1802,7 @@
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
@@ -2082,7 +2082,7 @@
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
@@ -2222,7 +2222,7 @@
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="F36" s="4" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -2397,7 +2397,7 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -2502,7 +2502,7 @@
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
@@ -2572,7 +2572,7 @@
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
@@ -2642,7 +2642,7 @@
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
@@ -2782,7 +2782,7 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -2922,7 +2922,7 @@
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
@@ -2957,7 +2957,7 @@
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
@@ -2992,7 +2992,7 @@
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
@@ -3027,7 +3027,7 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -3202,7 +3202,7 @@
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
@@ -3272,7 +3272,7 @@
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
@@ -3482,7 +3482,7 @@
         </is>
       </c>
       <c r="F70" s="4" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
         </is>
       </c>
       <c r="F72" s="4" t="n">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="F74" s="4" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
@@ -3657,7 +3657,7 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="F76" s="4" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
@@ -3762,7 +3762,7 @@
         </is>
       </c>
       <c r="F78" s="4" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
@@ -3832,7 +3832,7 @@
         </is>
       </c>
       <c r="F80" s="4" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
@@ -3902,7 +3902,7 @@
         </is>
       </c>
       <c r="F82" s="4" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
@@ -3972,7 +3972,7 @@
         </is>
       </c>
       <c r="F84" s="4" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="F85" s="4" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
@@ -4042,7 +4042,7 @@
         </is>
       </c>
       <c r="F86" s="4" t="n">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
@@ -4077,7 +4077,7 @@
         </is>
       </c>
       <c r="F87" s="4" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="F88" s="4" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="F89" s="4" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
@@ -4182,7 +4182,7 @@
         </is>
       </c>
       <c r="F90" s="4" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="F91" s="4" t="n">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
@@ -4252,7 +4252,7 @@
         </is>
       </c>
       <c r="F92" s="4" t="n">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="F93" s="4" t="n">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
@@ -4322,7 +4322,7 @@
         </is>
       </c>
       <c r="F94" s="4" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
@@ -4357,7 +4357,7 @@
         </is>
       </c>
       <c r="F95" s="4" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
@@ -4392,7 +4392,7 @@
         </is>
       </c>
       <c r="F96" s="4" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="F97" s="4" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="F98" s="4" t="n">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
@@ -4497,7 +4497,7 @@
         </is>
       </c>
       <c r="F99" s="4" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
@@ -4532,7 +4532,7 @@
         </is>
       </c>
       <c r="F100" s="4" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="F101" s="4" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
@@ -4602,7 +4602,7 @@
         </is>
       </c>
       <c r="F102" s="4" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="F103" s="4" t="n">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="G103" s="4" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         </is>
       </c>
       <c r="F104" s="4" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G104" s="4" t="inlineStr">
         <is>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="F105" s="4" t="n">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="G105" s="4" t="inlineStr">
         <is>
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="F106" s="4" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="F107" s="4" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="F108" s="4" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
@@ -4847,7 +4847,7 @@
         </is>
       </c>
       <c r="F109" s="4" t="n">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
@@ -4882,7 +4882,7 @@
         </is>
       </c>
       <c r="F110" s="4" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="F111" s="4" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
@@ -4952,7 +4952,7 @@
         </is>
       </c>
       <c r="F112" s="4" t="n">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="F113" s="4" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
@@ -5022,7 +5022,7 @@
         </is>
       </c>
       <c r="F114" s="4" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="G114" s="4" t="inlineStr">
         <is>
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="F115" s="4" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="G115" s="4" t="inlineStr">
         <is>
@@ -5092,7 +5092,7 @@
         </is>
       </c>
       <c r="F116" s="4" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G116" s="4" t="inlineStr">
         <is>
@@ -5127,7 +5127,7 @@
         </is>
       </c>
       <c r="F117" s="4" t="n">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="G117" s="4" t="inlineStr">
         <is>
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="F118" s="4" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="G118" s="4" t="inlineStr">
         <is>
@@ -5197,7 +5197,7 @@
         </is>
       </c>
       <c r="F119" s="4" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="G119" s="4" t="inlineStr">
         <is>
@@ -5232,7 +5232,7 @@
         </is>
       </c>
       <c r="F120" s="4" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G120" s="4" t="inlineStr">
         <is>
@@ -5267,7 +5267,7 @@
         </is>
       </c>
       <c r="F121" s="4" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G121" s="4" t="inlineStr">
         <is>
@@ -5302,7 +5302,7 @@
         </is>
       </c>
       <c r="F122" s="4" t="n">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="G122" s="4" t="inlineStr">
         <is>
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="F123" s="4" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G123" s="4" t="inlineStr">
         <is>
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="F124" s="4" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="G124" s="4" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
         </is>
       </c>
       <c r="F125" s="4" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="G125" s="4" t="inlineStr">
         <is>
@@ -5442,7 +5442,7 @@
         </is>
       </c>
       <c r="F126" s="4" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G126" s="4" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
         </is>
       </c>
       <c r="F127" s="4" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="G127" s="4" t="inlineStr">
         <is>
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="F128" s="4" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="G128" s="4" t="inlineStr">
         <is>
@@ -5547,7 +5547,7 @@
         </is>
       </c>
       <c r="F129" s="4" t="n">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="G129" s="4" t="inlineStr">
         <is>
@@ -5582,7 +5582,7 @@
         </is>
       </c>
       <c r="F130" s="4" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G130" s="4" t="inlineStr">
         <is>
@@ -5617,7 +5617,7 @@
         </is>
       </c>
       <c r="F131" s="4" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G131" s="4" t="inlineStr">
         <is>
@@ -5652,7 +5652,7 @@
         </is>
       </c>
       <c r="F132" s="4" t="n">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="G132" s="4" t="inlineStr">
         <is>
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="F133" s="4" t="n">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="G133" s="4" t="inlineStr">
         <is>
@@ -5757,7 +5757,7 @@
         </is>
       </c>
       <c r="F135" s="4" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G135" s="4" t="inlineStr">
         <is>
@@ -5792,7 +5792,7 @@
         </is>
       </c>
       <c r="F136" s="4" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="G136" s="4" t="inlineStr">
         <is>
@@ -5827,7 +5827,7 @@
         </is>
       </c>
       <c r="F137" s="4" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="G137" s="4" t="inlineStr">
         <is>
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="F138" s="4" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="G138" s="4" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
         </is>
       </c>
       <c r="F139" s="4" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="G139" s="4" t="inlineStr">
         <is>
@@ -5932,7 +5932,7 @@
         </is>
       </c>
       <c r="F140" s="4" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="G140" s="4" t="inlineStr">
         <is>
@@ -5967,7 +5967,7 @@
         </is>
       </c>
       <c r="F141" s="4" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="G141" s="4" t="inlineStr">
         <is>
@@ -6002,7 +6002,7 @@
         </is>
       </c>
       <c r="F142" s="4" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="G142" s="4" t="inlineStr">
         <is>
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="F143" s="4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="G143" s="4" t="inlineStr">
         <is>
@@ -6072,7 +6072,7 @@
         </is>
       </c>
       <c r="F144" s="4" t="n">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="G144" s="4" t="inlineStr">
         <is>
@@ -6107,7 +6107,7 @@
         </is>
       </c>
       <c r="F145" s="4" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G145" s="4" t="inlineStr">
         <is>
@@ -6142,7 +6142,7 @@
         </is>
       </c>
       <c r="F146" s="4" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="G146" s="4" t="inlineStr">
         <is>
@@ -6177,7 +6177,7 @@
         </is>
       </c>
       <c r="F147" s="4" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="G147" s="4" t="inlineStr">
         <is>
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="F148" s="4" t="n">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="G148" s="4" t="inlineStr">
         <is>
@@ -6247,7 +6247,7 @@
         </is>
       </c>
       <c r="F149" s="4" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G149" s="4" t="inlineStr">
         <is>
@@ -6282,7 +6282,7 @@
         </is>
       </c>
       <c r="F150" s="4" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="G150" s="4" t="inlineStr">
         <is>
@@ -6317,7 +6317,7 @@
         </is>
       </c>
       <c r="F151" s="4" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G151" s="4" t="inlineStr">
         <is>
@@ -6352,7 +6352,7 @@
         </is>
       </c>
       <c r="F152" s="4" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G152" s="4" t="inlineStr">
         <is>
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="F153" s="4" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="G153" s="4" t="inlineStr">
         <is>
@@ -6422,7 +6422,7 @@
         </is>
       </c>
       <c r="F154" s="4" t="n">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="G154" s="4" t="inlineStr">
         <is>
@@ -6457,7 +6457,7 @@
         </is>
       </c>
       <c r="F155" s="4" t="n">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="G155" s="4" t="inlineStr">
         <is>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="F156" s="4" t="n">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="G156" s="4" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         </is>
       </c>
       <c r="F157" s="4" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G157" s="4" t="inlineStr">
         <is>
@@ -6562,7 +6562,7 @@
         </is>
       </c>
       <c r="F158" s="4" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G158" s="4" t="inlineStr">
         <is>
@@ -6597,7 +6597,7 @@
         </is>
       </c>
       <c r="F159" s="4" t="n">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="G159" s="4" t="inlineStr">
         <is>
@@ -6632,7 +6632,7 @@
         </is>
       </c>
       <c r="F160" s="4" t="n">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="G160" s="4" t="inlineStr">
         <is>
@@ -6667,7 +6667,7 @@
         </is>
       </c>
       <c r="F161" s="4" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G161" s="4" t="inlineStr">
         <is>
@@ -6702,7 +6702,7 @@
         </is>
       </c>
       <c r="F162" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G162" s="4" t="inlineStr">
         <is>
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="F163" s="4" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G163" s="4" t="inlineStr">
         <is>
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="F164" s="4" t="n">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="G164" s="4" t="inlineStr">
         <is>
@@ -6807,7 +6807,7 @@
         </is>
       </c>
       <c r="F165" s="4" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G165" s="4" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
         </is>
       </c>
       <c r="F166" s="4" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G166" s="4" t="inlineStr">
         <is>
@@ -6877,7 +6877,7 @@
         </is>
       </c>
       <c r="F167" s="4" t="n">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G167" s="4" t="inlineStr">
         <is>
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="F168" s="4" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="G168" s="4" t="inlineStr">
         <is>
@@ -6947,7 +6947,7 @@
         </is>
       </c>
       <c r="F169" s="4" t="n">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="G169" s="4" t="inlineStr">
         <is>
@@ -6982,7 +6982,7 @@
         </is>
       </c>
       <c r="F170" s="4" t="n">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="G170" s="4" t="inlineStr">
         <is>
@@ -7017,7 +7017,7 @@
         </is>
       </c>
       <c r="F171" s="4" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G171" s="4" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
         </is>
       </c>
       <c r="F172" s="4" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G172" s="4" t="inlineStr">
         <is>
@@ -7122,7 +7122,7 @@
         </is>
       </c>
       <c r="F174" s="4" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="G174" s="4" t="inlineStr">
         <is>
@@ -7157,7 +7157,7 @@
         </is>
       </c>
       <c r="F175" s="4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G175" s="4" t="inlineStr">
         <is>
@@ -7192,7 +7192,7 @@
         </is>
       </c>
       <c r="F176" s="4" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="G176" s="4" t="inlineStr">
         <is>
@@ -7227,7 +7227,7 @@
         </is>
       </c>
       <c r="F177" s="4" t="n">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="G177" s="4" t="inlineStr">
         <is>
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="F178" s="4" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="G178" s="4" t="inlineStr">
         <is>
@@ -7297,7 +7297,7 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G179" s="4" t="inlineStr">
         <is>
@@ -7332,7 +7332,7 @@
         </is>
       </c>
       <c r="F180" s="4" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G180" s="4" t="inlineStr">
         <is>
@@ -7367,7 +7367,7 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="G181" s="4" t="inlineStr">
         <is>
@@ -7402,7 +7402,7 @@
         </is>
       </c>
       <c r="F182" s="4" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="G182" s="4" t="inlineStr">
         <is>
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="G183" s="4" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
         </is>
       </c>
       <c r="F184" s="4" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="G184" s="4" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="G185" s="4" t="inlineStr">
         <is>
@@ -7542,7 +7542,7 @@
         </is>
       </c>
       <c r="F186" s="4" t="n">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="G186" s="4" t="inlineStr">
         <is>
@@ -7577,7 +7577,7 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G187" s="4" t="inlineStr">
         <is>
@@ -7612,7 +7612,7 @@
         </is>
       </c>
       <c r="F188" s="4" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="G188" s="4" t="inlineStr">
         <is>
@@ -7647,7 +7647,7 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="G189" s="4" t="inlineStr">
         <is>
@@ -7682,7 +7682,7 @@
         </is>
       </c>
       <c r="F190" s="4" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G190" s="4" t="inlineStr">
         <is>
@@ -7717,7 +7717,7 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G191" s="4" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="G193" s="4" t="inlineStr">
         <is>
@@ -7822,7 +7822,7 @@
         </is>
       </c>
       <c r="F194" s="4" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="G194" s="4" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="G195" s="4" t="inlineStr">
         <is>
@@ -7892,7 +7892,7 @@
         </is>
       </c>
       <c r="F196" s="4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G196" s="4" t="inlineStr">
         <is>
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="G197" s="4" t="inlineStr">
         <is>
@@ -7962,7 +7962,7 @@
         </is>
       </c>
       <c r="F198" s="4" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="G198" s="4" t="inlineStr">
         <is>
@@ -7997,7 +7997,7 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G199" s="4" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
         </is>
       </c>
       <c r="F200" s="4" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G200" s="4" t="inlineStr">
         <is>
@@ -8067,7 +8067,7 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G201" s="4" t="inlineStr">
         <is>
@@ -8102,7 +8102,7 @@
         </is>
       </c>
       <c r="F202" s="4" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G202" s="4" t="inlineStr">
         <is>
@@ -8137,7 +8137,7 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G203" s="4" t="inlineStr">
         <is>
@@ -8172,7 +8172,7 @@
         </is>
       </c>
       <c r="F204" s="4" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="G204" s="4" t="inlineStr">
         <is>
@@ -8207,7 +8207,7 @@
         </is>
       </c>
       <c r="F205" s="4" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="G205" s="4" t="inlineStr">
         <is>
@@ -8242,7 +8242,7 @@
         </is>
       </c>
       <c r="F206" s="4" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="G206" s="4" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
         </is>
       </c>
       <c r="F207" s="4" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="G207" s="4" t="inlineStr">
         <is>
@@ -8312,7 +8312,7 @@
         </is>
       </c>
       <c r="F208" s="4" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G208" s="4" t="inlineStr">
         <is>
@@ -8347,7 +8347,7 @@
         </is>
       </c>
       <c r="F209" s="4" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G209" s="4" t="inlineStr">
         <is>
@@ -8382,7 +8382,7 @@
         </is>
       </c>
       <c r="F210" s="4" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="G210" s="4" t="inlineStr">
         <is>
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="F211" s="4" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G211" s="4" t="inlineStr">
         <is>
@@ -8452,7 +8452,7 @@
         </is>
       </c>
       <c r="F212" s="4" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="G212" s="4" t="inlineStr">
         <is>
@@ -8487,7 +8487,7 @@
         </is>
       </c>
       <c r="F213" s="4" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G213" s="4" t="inlineStr">
         <is>
@@ -8522,7 +8522,7 @@
         </is>
       </c>
       <c r="F214" s="4" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="G214" s="4" t="inlineStr">
         <is>
@@ -8557,7 +8557,7 @@
         </is>
       </c>
       <c r="F215" s="4" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G215" s="4" t="inlineStr">
         <is>
@@ -8592,7 +8592,7 @@
         </is>
       </c>
       <c r="F216" s="4" t="n">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="G216" s="4" t="inlineStr">
         <is>
@@ -8627,7 +8627,7 @@
         </is>
       </c>
       <c r="F217" s="4" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="G217" s="4" t="inlineStr">
         <is>
@@ -8662,7 +8662,7 @@
         </is>
       </c>
       <c r="F218" s="4" t="n">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="G218" s="4" t="inlineStr">
         <is>
@@ -8697,7 +8697,7 @@
         </is>
       </c>
       <c r="F219" s="4" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G219" s="4" t="inlineStr">
         <is>
@@ -8732,7 +8732,7 @@
         </is>
       </c>
       <c r="F220" s="4" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G220" s="4" t="inlineStr">
         <is>
@@ -8767,7 +8767,7 @@
         </is>
       </c>
       <c r="F221" s="4" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="G221" s="4" t="inlineStr">
         <is>
@@ -8802,7 +8802,7 @@
         </is>
       </c>
       <c r="F222" s="4" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G222" s="4" t="inlineStr">
         <is>
@@ -8837,7 +8837,7 @@
         </is>
       </c>
       <c r="F223" s="4" t="n">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G223" s="4" t="inlineStr">
         <is>
@@ -8872,7 +8872,7 @@
         </is>
       </c>
       <c r="F224" s="4" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="G224" s="4" t="inlineStr">
         <is>
@@ -8907,7 +8907,7 @@
         </is>
       </c>
       <c r="F225" s="4" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G225" s="4" t="inlineStr">
         <is>
@@ -8942,7 +8942,7 @@
         </is>
       </c>
       <c r="F226" s="4" t="n">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="G226" s="4" t="inlineStr">
         <is>
@@ -8977,7 +8977,7 @@
         </is>
       </c>
       <c r="F227" s="4" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G227" s="4" t="inlineStr">
         <is>
@@ -9012,7 +9012,7 @@
         </is>
       </c>
       <c r="F228" s="4" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="G228" s="4" t="inlineStr">
         <is>
@@ -9047,7 +9047,7 @@
         </is>
       </c>
       <c r="F229" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G229" s="4" t="inlineStr">
         <is>
@@ -9082,7 +9082,7 @@
         </is>
       </c>
       <c r="F230" s="4" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G230" s="4" t="inlineStr">
         <is>
@@ -9117,7 +9117,7 @@
         </is>
       </c>
       <c r="F231" s="4" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G231" s="4" t="inlineStr">
         <is>
@@ -9152,7 +9152,7 @@
         </is>
       </c>
       <c r="F232" s="4" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="G232" s="4" t="inlineStr">
         <is>
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="F233" s="4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G233" s="4" t="inlineStr">
         <is>
@@ -9222,7 +9222,7 @@
         </is>
       </c>
       <c r="F234" s="4" t="n">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="G234" s="4" t="inlineStr">
         <is>
@@ -9257,7 +9257,7 @@
         </is>
       </c>
       <c r="F235" s="4" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G235" s="4" t="inlineStr">
         <is>
@@ -9292,7 +9292,7 @@
         </is>
       </c>
       <c r="F236" s="4" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G236" s="4" t="inlineStr">
         <is>
@@ -9327,7 +9327,7 @@
         </is>
       </c>
       <c r="F237" s="4" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G237" s="4" t="inlineStr">
         <is>
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="F238" s="4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G238" s="4" t="inlineStr">
         <is>
@@ -9397,7 +9397,7 @@
         </is>
       </c>
       <c r="F239" s="4" t="n">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="G239" s="4" t="inlineStr">
         <is>
@@ -9432,7 +9432,7 @@
         </is>
       </c>
       <c r="F240" s="4" t="n">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="G240" s="4" t="inlineStr">
         <is>
@@ -9467,7 +9467,7 @@
         </is>
       </c>
       <c r="F241" s="4" t="n">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G241" s="4" t="inlineStr">
         <is>
@@ -9502,7 +9502,7 @@
         </is>
       </c>
       <c r="F242" s="4" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G242" s="4" t="inlineStr">
         <is>
@@ -9537,7 +9537,7 @@
         </is>
       </c>
       <c r="F243" s="4" t="n">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="G243" s="4" t="inlineStr">
         <is>
@@ -9572,7 +9572,7 @@
         </is>
       </c>
       <c r="F244" s="4" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="G244" s="4" t="inlineStr">
         <is>
@@ -9607,7 +9607,7 @@
         </is>
       </c>
       <c r="F245" s="4" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="G245" s="4" t="inlineStr">
         <is>
@@ -9642,7 +9642,7 @@
         </is>
       </c>
       <c r="F246" s="4" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G246" s="4" t="inlineStr">
         <is>
@@ -9677,7 +9677,7 @@
         </is>
       </c>
       <c r="F247" s="4" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G247" s="4" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="F248" s="4" t="n">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="G248" s="4" t="inlineStr">
         <is>
@@ -9747,7 +9747,7 @@
         </is>
       </c>
       <c r="F249" s="4" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="G249" s="4" t="inlineStr">
         <is>
@@ -9782,7 +9782,7 @@
         </is>
       </c>
       <c r="F250" s="4" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G250" s="4" t="inlineStr">
         <is>
@@ -9817,7 +9817,7 @@
         </is>
       </c>
       <c r="F251" s="4" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="G251" s="4" t="inlineStr">
         <is>
@@ -9852,7 +9852,7 @@
         </is>
       </c>
       <c r="F252" s="4" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="G252" s="4" t="inlineStr">
         <is>
@@ -9887,7 +9887,7 @@
         </is>
       </c>
       <c r="F253" s="4" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="G253" s="4" t="inlineStr">
         <is>
@@ -9922,7 +9922,7 @@
         </is>
       </c>
       <c r="F254" s="4" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G254" s="4" t="inlineStr">
         <is>
@@ -9957,7 +9957,7 @@
         </is>
       </c>
       <c r="F255" s="4" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="G255" s="4" t="inlineStr">
         <is>
@@ -9992,7 +9992,7 @@
         </is>
       </c>
       <c r="F256" s="4" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G256" s="4" t="inlineStr">
         <is>
@@ -10027,7 +10027,7 @@
         </is>
       </c>
       <c r="F257" s="4" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G257" s="4" t="inlineStr">
         <is>
@@ -10062,7 +10062,7 @@
         </is>
       </c>
       <c r="F258" s="4" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="G258" s="4" t="inlineStr">
         <is>
@@ -10097,7 +10097,7 @@
         </is>
       </c>
       <c r="F259" s="4" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="G259" s="4" t="inlineStr">
         <is>
@@ -10132,7 +10132,7 @@
         </is>
       </c>
       <c r="F260" s="4" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G260" s="4" t="inlineStr">
         <is>
@@ -10167,7 +10167,7 @@
         </is>
       </c>
       <c r="F261" s="4" t="n">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="G261" s="4" t="inlineStr">
         <is>
@@ -10202,7 +10202,7 @@
         </is>
       </c>
       <c r="F262" s="4" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G262" s="4" t="inlineStr">
         <is>
@@ -10237,7 +10237,7 @@
         </is>
       </c>
       <c r="F263" s="4" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G263" s="4" t="inlineStr">
         <is>
@@ -10272,7 +10272,7 @@
         </is>
       </c>
       <c r="F264" s="4" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="G264" s="4" t="inlineStr">
         <is>
@@ -10307,7 +10307,7 @@
         </is>
       </c>
       <c r="F265" s="4" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="G265" s="4" t="inlineStr">
         <is>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="F266" s="4" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G266" s="4" t="inlineStr">
         <is>
@@ -10377,7 +10377,7 @@
         </is>
       </c>
       <c r="F267" s="4" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G267" s="4" t="inlineStr">
         <is>
@@ -10412,7 +10412,7 @@
         </is>
       </c>
       <c r="F268" s="4" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G268" s="4" t="inlineStr">
         <is>
@@ -10447,7 +10447,7 @@
         </is>
       </c>
       <c r="F269" s="4" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G269" s="4" t="inlineStr">
         <is>
@@ -10482,7 +10482,7 @@
         </is>
       </c>
       <c r="F270" s="4" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G270" s="4" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         </is>
       </c>
       <c r="F271" s="4" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G271" s="4" t="inlineStr">
         <is>
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="F272" s="4" t="n">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="G272" s="4" t="inlineStr">
         <is>
@@ -10622,7 +10622,7 @@
         </is>
       </c>
       <c r="F274" s="4" t="n">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="G274" s="4" t="inlineStr">
         <is>
@@ -10657,7 +10657,7 @@
         </is>
       </c>
       <c r="F275" s="4" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="G275" s="4" t="inlineStr">
         <is>
@@ -10727,7 +10727,7 @@
         </is>
       </c>
       <c r="F277" s="4" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G277" s="4" t="inlineStr">
         <is>
@@ -10762,7 +10762,7 @@
         </is>
       </c>
       <c r="F278" s="4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G278" s="4" t="inlineStr">
         <is>
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="F279" s="4" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G279" s="4" t="inlineStr">
         <is>
@@ -10832,7 +10832,7 @@
         </is>
       </c>
       <c r="F280" s="4" t="n">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="G280" s="4" t="inlineStr">
         <is>
@@ -10867,7 +10867,7 @@
         </is>
       </c>
       <c r="F281" s="4" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G281" s="4" t="inlineStr">
         <is>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="F282" s="4" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G282" s="4" t="inlineStr">
         <is>
@@ -10937,7 +10937,7 @@
         </is>
       </c>
       <c r="F283" s="4" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="G283" s="4" t="inlineStr">
         <is>
@@ -10972,7 +10972,7 @@
         </is>
       </c>
       <c r="F284" s="4" t="n">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G284" s="4" t="inlineStr">
         <is>
@@ -11007,7 +11007,7 @@
         </is>
       </c>
       <c r="F285" s="4" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="G285" s="4" t="inlineStr">
         <is>
@@ -11042,7 +11042,7 @@
         </is>
       </c>
       <c r="F286" s="4" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="G286" s="4" t="inlineStr">
         <is>
@@ -11077,7 +11077,7 @@
         </is>
       </c>
       <c r="F287" s="4" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="G287" s="4" t="inlineStr">
         <is>
@@ -11112,7 +11112,7 @@
         </is>
       </c>
       <c r="F288" s="4" t="n">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="G288" s="4" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
         </is>
       </c>
       <c r="F289" s="4" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G289" s="4" t="inlineStr">
         <is>
@@ -11182,7 +11182,7 @@
         </is>
       </c>
       <c r="F290" s="4" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G290" s="4" t="inlineStr">
         <is>
@@ -11217,7 +11217,7 @@
         </is>
       </c>
       <c r="F291" s="4" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G291" s="4" t="inlineStr">
         <is>
@@ -11252,7 +11252,7 @@
         </is>
       </c>
       <c r="F292" s="4" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="G292" s="4" t="inlineStr">
         <is>
@@ -11287,7 +11287,7 @@
         </is>
       </c>
       <c r="F293" s="4" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G293" s="4" t="inlineStr">
         <is>
@@ -11322,7 +11322,7 @@
         </is>
       </c>
       <c r="F294" s="4" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="G294" s="4" t="inlineStr">
         <is>
@@ -11357,7 +11357,7 @@
         </is>
       </c>
       <c r="F295" s="4" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="G295" s="4" t="inlineStr">
         <is>
@@ -11392,7 +11392,7 @@
         </is>
       </c>
       <c r="F296" s="4" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="G296" s="4" t="inlineStr">
         <is>
@@ -11427,7 +11427,7 @@
         </is>
       </c>
       <c r="F297" s="4" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="G297" s="4" t="inlineStr">
         <is>
@@ -11462,7 +11462,7 @@
         </is>
       </c>
       <c r="F298" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G298" s="4" t="inlineStr">
         <is>
@@ -11497,7 +11497,7 @@
         </is>
       </c>
       <c r="F299" s="4" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G299" s="4" t="inlineStr">
         <is>
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="F300" s="4" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="G300" s="4" t="inlineStr">
         <is>
@@ -11567,7 +11567,7 @@
         </is>
       </c>
       <c r="F301" s="4" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="G301" s="4" t="inlineStr">
         <is>
@@ -11978,7 +11978,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29 02:58:15</t>
+          <t>2026-07-29 03:01:57</t>
         </is>
       </c>
     </row>

</xml_diff>